<commit_message>
Prijata posta: Excel zoznam - zmazany Bonn, precislovanie od 01
</commit_message>
<xml_diff>
--- a/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
+++ b/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -560,14 +560,14 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Scan_2024_03_22_BONN.pdf</t>
+          <t>zaloba_proti_Telekomu_DE_original_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>01_22.03.2024_Scan_Schreiben_Bonn_Deutsche_Telekom_DE_GH.pdf</t>
+          <t>01_02.10.2024_Klage_gegen_Telekom_und_Schufa_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -577,23 +577,23 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>22.03.2024</t>
+          <t>02.10.2024</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Sken – list z Bonnu (pravdepodobne Deutsche Telekom AG)</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Deutsche Telekom AG (overiť)</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
+          <t>Žaloba proti Deutsche Telekom AG a SCHUFA Holding AG</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>FES</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Sken; odosielateľa a predmet OVERIŤ – ak nie je Telekom, popis upravím</t>
+          <t>VLASTNÉ podanie Petra – patrí do odoslanej pošty; tu je len kópia. Potvrď či nechať v došlej.</t>
         </is>
       </c>
     </row>
@@ -603,14 +603,14 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>zaloba_proti_Telekomu_DE_original_DE_GH.pdf</t>
+          <t>Oznamenie_o_prideleni_Akten_23_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>02_02.10.2024_Klage_gegen_Telekom_und_Schufa_DE_GH.pdf</t>
+          <t>02_08.10.2024_Anschreiben_und_Aktenzuteilung_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -620,23 +620,19 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>02.10.2024</t>
+          <t>08.10.2024</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Žaloba proti Deutsche Telekom AG a SCHUFA Holding AG</t>
+          <t>Sprievodný list + oznámenie o pridelení spisu</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>FES</t>
-        </is>
-      </c>
+      <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>VLASTNÉ podanie Petra – patrí do odoslanej pošty; tu je len kópia. Potvrď či nechať v došlej.</t>
+          <t>→ klon P01</t>
         </is>
       </c>
     </row>
@@ -646,14 +642,14 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Oznamenie_o_prideleni_Akten_23_O_2699_24_DE_GH.pdf</t>
+          <t>sud_LA_upozornenie_dokumenty_nepredstavuju_pravne_ucinne_navrhy_DE_original.pdf</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>03_08.10.2024_Anschreiben_und_Aktenzuteilung_DE_GH.pdf</t>
+          <t>03_10.10.2024_Hinweis_Anwaltszwang_par78_ZPO_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -663,19 +659,19 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>08.10.2024</t>
+          <t>10.10.2024</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Sprievodný list + oznámenie o pridelení spisu</t>
+          <t>Upozornenie: podania bez advokáta nie sú právne účinné (§ 78 ZPO)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>→ klon P01</t>
+          <t>→ klon P02</t>
         </is>
       </c>
     </row>
@@ -685,14 +681,14 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>sud_LA_upozornenie_dokumenty_nepredstavuju_pravne_ucinne_navrhy_DE_original.pdf</t>
+          <t>anwaltliche_Vertretung_23_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>04_10.10.2024_Hinweis_Anwaltszwang_par78_ZPO_DE_GH.pdf</t>
+          <t>04_17.10.2024_Anwaltliche_Vertretung_Latham_Watkins_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -702,19 +698,23 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>10.10.2024</t>
+          <t>17.10.2024</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Upozornenie: podania bez advokáta nie sú právne účinné (§ 78 ZPO)</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+          <t>Oznámenie advokátskeho zastúpenia žalovaných</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Latham &amp; Watkins LLP</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>→ klon P02</t>
+          <t>1-stranový sken (Office Lens)</t>
         </is>
       </c>
     </row>
@@ -724,14 +724,14 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>anwaltliche_Vertretung_23_O_2699_24_DE_GH.pdf</t>
+          <t>6_11_KOSTENRECHNUNG_spis_23_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>05_17.10.2024_Anwaltliche_Vertretung_Latham_Watkins_DE_GH.pdf</t>
+          <t>05_06.11.2024_Kostenrechnung_LJK_Bamberg_17643_EUR_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -741,23 +741,23 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>17.10.2024</t>
+          <t>06.11.2024</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Oznámenie advokátskeho zastúpenia žalovaných</t>
+          <t>Kostenrechnung – vyúčtovanie súdneho poplatku 17 643 € (hodnota sporu 1 000 000 €)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Latham &amp; Watkins LLP</t>
+          <t>Landesjustizkasse Bamberg</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>1-stranový sken (Office Lens)</t>
+          <t>KV-GKG 1210, sadzba 3,0; poučenie o Erinnerung na 2. strane</t>
         </is>
       </c>
     </row>
@@ -767,14 +767,14 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>6_11_KOSTENRECHNUNG_spis_23_O_2699_24_DE_GH.pdf</t>
+          <t>Merged_LATHAM_a_WATKINS_ich_reakcia_na_sude_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>06_06.11.2024_Kostenrechnung_LJK_Bamberg_17643_EUR_DE_GH.pdf</t>
+          <t>06_20.11.2024_Stellungnahme_Latham_Watkins_PKH_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -784,23 +784,27 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>06.11.2024</t>
+          <t>20.11.2024</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Kostenrechnung – vyúčtovanie súdneho poplatku 17 643 € (hodnota sporu 1 000 000 €)</t>
+          <t>Stellungnahme Latham &amp; Watkins k návrhu na oslobodenie od trov (za SCHUFA Holding AG)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Landesjustizkasse Bamberg</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
+          <t>Latham &amp; Watkins LLP (za SCHUFA Holding AG)</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>QES</t>
+        </is>
+      </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>KV-GKG 1210, sadzba 3,0; poučenie o Erinnerung na 2. strane</t>
+          <t>Petrov Word – str. 5–10 zlúčeného; → klon P10; pravý beA originál v repe chýba</t>
         </is>
       </c>
     </row>
@@ -810,14 +814,14 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Merged_LATHAM_a_WATKINS_ich_reakcia_na_sude_DE_GH.pdf</t>
+          <t>Beshlus_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>07_20.11.2024_Stellungnahme_Latham_Watkins_PKH_DE_GH.pdf</t>
+          <t>07_21.11.2024_Beschluss_PKH_abgelehnt_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -827,27 +831,19 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>20.11.2024</t>
+          <t>21.11.2024</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Stellungnahme Latham &amp; Watkins k návrhu na oslobodenie od trov (za SCHUFA Holding AG)</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Latham &amp; Watkins LLP (za SCHUFA Holding AG)</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>QES</t>
-        </is>
-      </c>
+          <t>Beschluss – zamietnutie oslobodenia od trov (PKH) + poučenie o opravných prostriedkoch</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Petrov Word – str. 5–10 zlúčeného; → klon P10; pravý beA originál v repe chýba</t>
+          <t>Sudkyňa Pfenninger; → klon P09</t>
         </is>
       </c>
     </row>
@@ -857,14 +853,14 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Beshlus_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
+          <t>22_11_24_odpoved_na_prozeskostenhilfeDE_originalDE_GH.pdf</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>08_21.11.2024_Beschluss_PKH_abgelehnt_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
+          <t>08_22.11.2024_Schreiben_zur_Prozesskostenhilfe_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -874,19 +870,19 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>21.11.2024</t>
+          <t>22.11.2024</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Beschluss – zamietnutie oslobodenia od trov (PKH) + poučenie o opravných prostriedkoch</t>
+          <t>List / odpoveď vo veci oslobodenia od trov (PKH)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Sudkyňa Pfenninger; → klon P09</t>
+          <t>Predmet OVERIŤ – upresním popis</t>
         </is>
       </c>
     </row>
@@ -896,14 +892,14 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>22_11_24_odpoved_na_prozeskostenhilfeDE_originalDE_GH.pdf</t>
+          <t>Kostennachricht_Bamberg_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>09_22.11.2024_Schreiben_zur_Prozesskostenhilfe_DE_GH.pdf</t>
+          <t>09_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -913,19 +909,23 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>22.11.2024</t>
+          <t>27.11.2024</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>List / odpoveď vo veci oslobodenia od trov (PKH)</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+          <t>Kostennachricht – oznámenie o trovách</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Landesjustizkasse Bamberg</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Predmet OVERIŤ – upresním popis</t>
+          <t>→ klon P07; dátum OVERIŤ</t>
         </is>
       </c>
     </row>
@@ -935,14 +935,14 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Kostennachricht_Bamberg_DE_GH.pdf</t>
+          <t>Antrag_auf_Erlass_einer_einstweiligen_Verfugung_ORIGINAL_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>10_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
+          <t>10_11.12.2024_Antrag_einstweilige_Verfuegung_Original_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -952,23 +952,23 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>27.11.2024</t>
+          <t>11.12.2024</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Kostennachricht – oznámenie o trovách</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Landesjustizkasse Bamberg</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
+          <t>Návrh na vydanie predbežného opatrenia (originál)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>QES</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>→ klon P07; dátum OVERIŤ</t>
+          <t>VLASTNÉ podanie Petra – patrí do odoslanej pošty; tu je len kópia. Potvrď.</t>
         </is>
       </c>
     </row>
@@ -978,14 +978,14 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Antrag_auf_Erlass_einer_einstweiligen_Verfugung_ORIGINAL_DE_GH.pdf</t>
+          <t>reklamacia_QES_zo_sudu_LA_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr"/>
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>11_11.12.2024_Antrag_einstweilige_Verfuegung_Original_DE_GH.pdf</t>
+          <t>11_12.12.2024_Hinweis_Signatur_nicht_pruefbar_par130d_ZPO_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -995,23 +995,19 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>11.12.2024</t>
+          <t>12.12.2024</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Návrh na vydanie predbežného opatrenia (originál)</t>
+          <t>Oznámenie súdu k forme podania – nemožno overiť podpis (§ 130d ZPO)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>QES</t>
-        </is>
-      </c>
+      <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>VLASTNÉ podanie Petra – patrí do odoslanej pošty; tu je len kópia. Potvrď.</t>
+          <t>Forma podania</t>
         </is>
       </c>
     </row>
@@ -1021,14 +1017,14 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>reklamacia_QES_zo_sudu_LA_DE_GH.pdf</t>
+          <t>vo_veci_Schufa_Holding_AG_a_Deutsche_Telekom_AG_DE_GHoriginal.pdf</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>12_12.12.2024_Hinweis_Signatur_nicht_pruefbar_par130d_ZPO_DE_GH.pdf</t>
+          <t>12_16.12.2024_Schreiben_in_Sachen_Schufa_Telekom_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1038,19 +1034,19 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>12.12.2024</t>
+          <t>16.12.2024</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Oznámenie súdu k forme podania – nemožno overiť podpis (§ 130d ZPO)</t>
+          <t>List súdu vo veci SCHUFA Holding AG a Deutsche Telekom AG</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Forma podania</t>
+          <t>1-stranový sken (Office Lens); dátum z metadát skenu, OVERIŤ</t>
         </is>
       </c>
     </row>
@@ -1060,14 +1056,14 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>vo_veci_Schufa_Holding_AG_a_Deutsche_Telekom_AG_DE_GHoriginal.pdf</t>
+          <t>sud_LA_zmena_spisovej_znacky_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
       <c r="D14" s="3" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>13_16.12.2024_Schreiben_in_Sachen_Schufa_Telekom_DE_GH.pdf</t>
+          <t>13_07.01.2025_Aenderung_Aktenzeichen_91_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1077,19 +1073,19 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>16.12.2024</t>
+          <t>07.01.2025</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>List súdu vo veci SCHUFA Holding AG a Deutsche Telekom AG</t>
+          <t>Zmena spisovej značky 23 O 2699/24 → 91 O 2699/24</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>1-stranový sken (Office Lens); dátum z metadát skenu, OVERIŤ</t>
+          <t>Senát 526 → 416; → klon P05</t>
         </is>
       </c>
     </row>
@@ -1099,14 +1095,14 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>sud_LA_zmena_spisovej_znacky_DE_GH.pdf</t>
+          <t>2025_01_22_LG_Landshut_potvrdenie_prijatia_emailu_20_01_2025_DE_original.pdf</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>14_07.01.2025_Aenderung_Aktenzeichen_91_O_2699_24_DE_GH.pdf</t>
+          <t>14_22.01.2025_Empfangsbestaetigung_Email_20_01_2025_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1116,56 +1112,17 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>07.01.2025</t>
+          <t>22.01.2025</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Zmena spisovej značky 23 O 2699/24 → 91 O 2699/24</t>
+          <t>Potvrdenie prijatia e-mailu z 20.01.2025 (na sudcovský príkaz)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Senát 526 → 416; → klon P05</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>2025_01_22_LG_Landshut_potvrdenie_prijatia_emailu_20_01_2025_DE_original.pdf</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>15_22.01.2025_Empfangsbestaetigung_Email_20_01_2025_DE_GH.pdf</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>prijaté</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>22.01.2025</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Potvrdenie prijatia e-mailu z 20.01.2025 (na sudcovský príkaz)</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>→ klon P08</t>
         </is>

</xml_diff>

<commit_message>
Prijata posta: Excel - opravene datumy/predmety z obsahu, cislovanie 01-14
</commit_message>
<xml_diff>
--- a/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
+++ b/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
@@ -486,15 +486,15 @@
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -505,7 +505,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Pôvodný názov súboru (starý, z repa/disku)</t>
+          <t>Pôvodný názov (zdroj v repe)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -520,7 +520,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Nový názov (návrh Claude) — repo aj OneDrive</t>
+          <t>Nový názov (finálny, repo aj OneDrive)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Poznámka</t>
+          <t>Poznámka / klon</t>
         </is>
       </c>
     </row>
@@ -560,14 +560,14 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>zaloba_proti_Telekomu_DE_original_DE_GH.pdf</t>
+          <t>Oznamenie_o_prideleni_Akten_23_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>01_02.10.2024_Klage_gegen_Telekom_und_Schufa_DE_GH.pdf</t>
+          <t>01_08.10.2024_Anschreiben_beglaubigte_Abschrift_Beschluss_07.10.2024_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -577,23 +577,19 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>02.10.2024</t>
+          <t>08.10.2024</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Žaloba proti Deutsche Telekom AG a SCHUFA Holding AG</t>
+          <t>Sprievodný list + overený odpis uznesenia zo 07.10.2024 (hodnota sporu 1 000 000 €)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>FES</t>
-        </is>
-      </c>
+      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>VLASTNÉ podanie Petra – patrí do odoslanej pošty; tu je len kópia. Potvrď či nechať v došlej.</t>
+          <t>→ klon P01</t>
         </is>
       </c>
     </row>
@@ -603,14 +599,14 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Oznamenie_o_prideleni_Akten_23_O_2699_24_DE_GH.pdf</t>
+          <t>anwaltliche_Vertretung_23_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>02_08.10.2024_Anschreiben_und_Aktenzuteilung_DE_GH.pdf</t>
+          <t>02_10.10.2024_Hinweis_Anwaltszwang_par78_ZPO_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -620,19 +616,19 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>08.10.2024</t>
+          <t>10.10.2024</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Sprievodný list + oznámenie o pridelení spisu</t>
+          <t>Upozornenie § 78 ZPO: bez advokáta nemožno doručiť (žaloba aj e-mail prijaté)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>→ klon P01</t>
+          <t>→ klon P02</t>
         </is>
       </c>
     </row>
@@ -642,14 +638,14 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>sud_LA_upozornenie_dokumenty_nepredstavuju_pravne_ucinne_navrhy_DE_original.pdf</t>
+          <t>zaloba_proti_Telekomu_DE_original_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>03_10.10.2024_Hinweis_Anwaltszwang_par78_ZPO_DE_GH.pdf</t>
+          <t>03_06.11.2024_Verfuegung_Klageentwurf_an_Beklagte_PKH_Frist_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -659,19 +655,19 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>10.10.2024</t>
+          <t>06.11.2024</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Upozornenie: podania bez advokáta nie sú právne účinné (§ 78 ZPO)</t>
+          <t>Verfügung: návrh žaloby sa posiela žalovaným; lehota na PKH-stanovisko predĺžená do 20.11.2024</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>→ klon P02</t>
+          <t>Súdny list (nie Petrova žaloba); v prílohe Klageentwurf z 02.10</t>
         </is>
       </c>
     </row>
@@ -681,14 +677,14 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>anwaltliche_Vertretung_23_O_2699_24_DE_GH.pdf</t>
+          <t>6_11_KOSTENRECHNUNG_spis_23_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>04_17.10.2024_Anwaltliche_Vertretung_Latham_Watkins_DE_GH.pdf</t>
+          <t>04_06.11.2024_Kostenrechnung_LJK_Bamberg_17643_EUR_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -698,25 +694,21 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>17.10.2024</t>
+          <t>06.11.2024</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Oznámenie advokátskeho zastúpenia žalovaných</t>
+          <t>Kostenrechnung – súdny poplatok 17 643 € (KV-GKG 1210, sadzba 3,0)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Latham &amp; Watkins LLP</t>
+          <t>Landesjustizkasse Bamberg</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>1-stranový sken (Office Lens)</t>
-        </is>
-      </c>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -724,14 +716,14 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>6_11_KOSTENRECHNUNG_spis_23_O_2699_24_DE_GH.pdf</t>
+          <t>Merged_LATHAM_a_WATKINS_ich_reakcia_na_sude_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>05_06.11.2024_Kostenrechnung_LJK_Bamberg_17643_EUR_DE_GH.pdf</t>
+          <t>05_20.11.2024_Stellungnahme_Latham_Watkins_PKH_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -741,23 +733,27 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>06.11.2024</t>
+          <t>20.11.2024</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Kostenrechnung – vyúčtovanie súdneho poplatku 17 643 € (hodnota sporu 1 000 000 €)</t>
+          <t>Stellungnahme Latham &amp; Watkins k PKH (za SCHUFA Holding AG)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Landesjustizkasse Bamberg</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
+          <t>Latham &amp; Watkins LLP (za SCHUFA Holding AG)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>QES</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>KV-GKG 1210, sadzba 3,0; poučenie o Erinnerung na 2. strane</t>
+          <t>→ klon P10; Petrov Word (str. 5–10 zlúčeného); pravý beA originál chýba</t>
         </is>
       </c>
     </row>
@@ -767,14 +763,14 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Merged_LATHAM_a_WATKINS_ich_reakcia_na_sude_DE_GH.pdf</t>
+          <t>Beshlus_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>06_20.11.2024_Stellungnahme_Latham_Watkins_PKH_DE_GH.pdf</t>
+          <t>06_21.11.2024_Beschluss_PKH_abgelehnt_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -784,27 +780,19 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>20.11.2024</t>
+          <t>21.11.2024</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Stellungnahme Latham &amp; Watkins k návrhu na oslobodenie od trov (za SCHUFA Holding AG)</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Latham &amp; Watkins LLP (za SCHUFA Holding AG)</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>QES</t>
-        </is>
-      </c>
+          <t>Beschluss: PKH zamietnutá + poučenie o opravných prostriedkoch (sudkyňa Pfenninger)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Petrov Word – str. 5–10 zlúčeného; → klon P10; pravý beA originál v repe chýba</t>
+          <t>→ klon P09</t>
         </is>
       </c>
     </row>
@@ -814,14 +802,14 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Beshlus_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
+          <t>22_11_24_odpoved_na_prozeskostenhilfeDE_originalDE_GH.pdf</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>07_21.11.2024_Beschluss_PKH_abgelehnt_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
+          <t>07_21.11.2024_Beschluss_PKH_beglaubigte_Abschrift_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -836,14 +824,14 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Beschluss – zamietnutie oslobodenia od trov (PKH) + poučenie o opravných prostriedkoch</t>
+          <t>Beschluss PKH – overený odpis (9 s.)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Sudkyňa Pfenninger; → klon P09</t>
+          <t>DUPLICITA k č. 06 (ten istý Beschluss z 21.11) – zvážiť ponechať/zmazať</t>
         </is>
       </c>
     </row>
@@ -853,14 +841,14 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>22_11_24_odpoved_na_prozeskostenhilfeDE_originalDE_GH.pdf</t>
+          <t>Kostennachricht_Bamberg_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>08_22.11.2024_Schreiben_zur_Prozesskostenhilfe_DE_GH.pdf</t>
+          <t>08_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -870,19 +858,23 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>22.11.2024</t>
+          <t>27.11.2024</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>List / odpoveď vo veci oslobodenia od trov (PKH)</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
+          <t>Kostennachricht – oznámenie o trovách (poučenie o Erinnerung)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Landesjustizkasse Bamberg</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Predmet OVERIŤ – upresním popis</t>
+          <t>→ klon P07</t>
         </is>
       </c>
     </row>
@@ -892,14 +884,14 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Kostennachricht_Bamberg_DE_GH.pdf</t>
+          <t>vo_veci_Schufa_Holding_AG_a_Deutsche_Telekom_AG_DE_GHoriginal.pdf</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>09_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
+          <t>09_03.12.2024_Anregung_Ruecknahme_Beschwerde_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -909,23 +901,19 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>27.11.2024</t>
+          <t>03.12.2024</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Kostennachricht – oznámenie o trovách</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Landesjustizkasse Bamberg</t>
-        </is>
-      </c>
+          <t>Súd navrhuje späťvzatie sťažnosti (rozhodnutie z 21.11 doručené 26.11; sťažnosť z 25.11)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>→ klon P07; dátum OVERIŤ</t>
+          <t>→ klon P06</t>
         </is>
       </c>
     </row>
@@ -942,7 +930,7 @@
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>10_11.12.2024_Antrag_einstweilige_Verfuegung_Original_DE_GH.pdf</t>
+          <t>10_12.12.2024_Hinweis_Beschwerde_und_eV_nur_schriftlich_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -952,23 +940,19 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>11.12.2024</t>
+          <t>12.12.2024</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Návrh na vydanie predbežného opatrenia (originál)</t>
+          <t>Súdny list: Beschwerde 07.12 a návrh na eV 11.12 prišli e-mailom, prípustné len písomne</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>QES</t>
-        </is>
-      </c>
+      <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>VLASTNÉ podanie Petra – patrí do odoslanej pošty; tu je len kópia. Potvrď.</t>
+          <t>Súdny list (nie Petrov návrh na eV)</t>
         </is>
       </c>
     </row>
@@ -985,7 +969,7 @@
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>11_12.12.2024_Hinweis_Signatur_nicht_pruefbar_par130d_ZPO_DE_GH.pdf</t>
+          <t>11_17.12.2024_Hinweis_Form_par130a_Post_oder_QES_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -995,19 +979,19 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>12.12.2024</t>
+          <t>17.12.2024</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Oznámenie súdu k forme podania – nemožno overiť podpis (§ 130d ZPO)</t>
+          <t>Poučenie o forme § 130a: poštou s vlastnoručným podpisom ALEBO elektronicky s QES</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Forma podania</t>
+          <t>→ klon P03 (JADRO argumentu)</t>
         </is>
       </c>
     </row>
@@ -1017,14 +1001,14 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>vo_veci_Schufa_Holding_AG_a_Deutsche_Telekom_AG_DE_GHoriginal.pdf</t>
+          <t>sud_LA_upozornenie_dokumenty_nepredstavuju_pravne_ucinne_navrhy_DE_original.pdf</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>12_16.12.2024_Schreiben_in_Sachen_Schufa_Telekom_DE_GH.pdf</t>
+          <t>12_23.12.2024_Hinweis_Email_keine_formwirksamen_Antraege_nur_Post_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1034,19 +1018,19 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>16.12.2024</t>
+          <t>23.12.2024</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>List súdu vo veci SCHUFA Holding AG a Deutsche Telekom AG</t>
+          <t>E-maily nie sú formálne platné návrhy; kým nepodá poštou, e-maily sa už nebudú spracúvať</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>1-stranový sken (Office Lens); dátum z metadát skenu, OVERIŤ</t>
+          <t>→ klon P04 (JADRO argumentu – odvolanie návodu)</t>
         </is>
       </c>
     </row>
@@ -1078,14 +1062,14 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Zmena spisovej značky 23 O 2699/24 → 91 O 2699/24</t>
+          <t>Zmena spisovej značky 23 O 2699/24 → 91 O 2699/24 (senát 526 → 416)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Senát 526 → 416; → klon P05</t>
+          <t>→ klon P05</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1108,7 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>→ klon P08</t>
+          <t>→ klon P08; sken</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1149,7 +1133,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Ako tabuľku vyplniť / premenovať</t>
+          <t>Zoznam – prijatá (došlá) pošta, kauza LG Landshut 23 O 2699/24 → 91 O 2699/24</t>
         </is>
       </c>
       <c r="B1" s="6" t="inlineStr"/>
@@ -1161,120 +1145,84 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Zelený stĺpec E — Nový názov</t>
+          <t>Dôležité</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>NÁVRH Claude: NN_DD.MM.RRRR_popis_bez_diakritiky_DE_GH.pdf. Číslované chronologicky (01 = najstarší). Po tvojom OK premenujem v repe; ty premenuj rovnako na OneDrive.</t>
+          <t>Dátumy a predmety sú OVERENÉ z obsahu dokumentov (nie z názvov). Predošlé číslovanie bolo podľa nepresných názvov – opravené.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Žlté stĺpce (C, D)</t>
+          <t>Zelený stĺpec E</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Vypĺňa Peter (cesta na disku, OneDrive odkaz). Ostatné predvyplnil Claude.</t>
+          <t>Finálny názov v repe aj na OneDrive: NN_DD.MM.RRRR_popis_bez_diakritiky_DE_GH.pdf, chronologicky.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Stĺpec B</t>
+          <t>Žlté C, D</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Starý (pôvodný) názov v repe/na disku — podľa neho spáruj a premenuj na E.</t>
+          <t>Vypĺňa Peter (cesta na disku, OneDrive odkaz).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>F — Smer</t>
+          <t>Stĺpec B</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Tu všetko «prijaté» (došlá pošta). Riadky 02 a 11 sú Petrove vlastné podania (kópie) — potvrď, či majú ostať v došlej.</t>
+          <t>Pôvodný zdrojový názov v repe – podľa neho spáruj a premenuj na E.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>G — Dátum</t>
+          <t>Duplicita</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>DD.MM.RRRR. «OVERIŤ» v poznámke = dátum/predmet ešte potvrdiť.</t>
+          <t>č. 06 a 07 sú ten istý Beschluss z 21.11.2024 (rôzna dĺžka). Rozhodnúť, či ponechať oba.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>H — Predmet</t>
+          <t>Klony</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Krátky SK predmet — Claude preloží do 9 jazykov na karte.</t>
+          <t>Mapovanie na viacjazyčné klony P01–P10 je v stĺpci Poznámka. Klony sa premenujú na P + číslo originálu (samostatný krok).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>I — Orgán</t>
+          <t>Cesta na disku</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Len ak iný než Landgericht Landshut (Bamberg, Latham &amp; Watkins, Deutsche Telekom).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>J — Podpis</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>QES / FES / prázdne.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Cesta na disku</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
           <t>d:\OneDrive - Peter Ferenc Foxpro\Dokumenty\Bundesbeauftragte\Súd Landshut Telekom žaloba\Pošta\Došlá pošta\GH\</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Pozn.</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Popisy sú v nemčine (dokumenty sú DE originály). Ak chceš SK popisy, poviem a prepíšem. Klony P01–P10 sú odvodené výstupy, nepremenúvajú sa týmto.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register prijate: zmazany riadok 06 (duplikat 07), klony zosynchronizovane P01-P14 (P06 medzera)
</commit_message>
<xml_diff>
--- a/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
+++ b/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -667,7 +667,7 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Súdny list (nie Petrova žaloba); v prílohe Klageentwurf z 02.10</t>
+          <t>Súdny list (nie Petrova žaloba); v prílohe Klageentwurf z 02.10 → klon P03</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,11 @@
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>→ klon P04</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -753,24 +757,24 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>→ klon P10; Petrov Word (str. 5–10 zlúčeného); pravý beA originál chýba</t>
+          <t>→ klon P05; Petrov Word (str. 5–10 zlúčeného); pravý beA originál chýba</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Beshlus_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
+          <t>22_11_24_odpoved_na_prozeskostenhilfeDE_originalDE_GH.pdf</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>06_21.11.2024_Beschluss_PKH_abgelehnt_Rechtsbehelfsbelehrung_DE_GH.pdf</t>
+          <t>07_21.11.2024_Beschluss_PKH_beglaubigte_Abschrift_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -785,31 +789,31 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Beschluss: PKH zamietnutá + poučenie o opravných prostriedkoch (sudkyňa Pfenninger)</t>
+          <t>Beschluss PKH – overený odpis (9 s.)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>→ klon P09</t>
+          <t>→ klon P07; beglaubigte Abschrift (9 str.); originál Beschlussu 21.11 (06 zmazaný ako duplikát)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>22_11_24_odpoved_na_prozeskostenhilfeDE_originalDE_GH.pdf</t>
+          <t>Kostennachricht_Bamberg_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>07_21.11.2024_Beschluss_PKH_beglaubigte_Abschrift_DE_GH.pdf</t>
+          <t>08_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -819,36 +823,40 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>21.11.2024</t>
+          <t>27.11.2024</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Beschluss PKH – overený odpis (9 s.)</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+          <t>Kostennachricht – oznámenie o trovách (poučenie o Erinnerung)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Landesjustizkasse Bamberg</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>DUPLICITA k č. 06 (ten istý Beschluss z 21.11) – zvážiť ponechať/zmazať</t>
+          <t>→ klon P08</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Kostennachricht_Bamberg_DE_GH.pdf</t>
+          <t>vo_veci_Schufa_Holding_AG_a_Deutsche_Telekom_AG_DE_GHoriginal.pdf</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>08_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
+          <t>09_03.12.2024_Anregung_Ruecknahme_Beschwerde_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -858,40 +866,36 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>27.11.2024</t>
+          <t>03.12.2024</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Kostennachricht – oznámenie o trovách (poučenie o Erinnerung)</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Landesjustizkasse Bamberg</t>
-        </is>
-      </c>
+          <t>Súd navrhuje späťvzatie sťažnosti (rozhodnutie z 21.11 doručené 26.11; sťažnosť z 25.11)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>→ klon P07</t>
+          <t>→ klon P09</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>vo_veci_Schufa_Holding_AG_a_Deutsche_Telekom_AG_DE_GHoriginal.pdf</t>
+          <t>Antrag_auf_Erlass_einer_einstweiligen_Verfugung_ORIGINAL_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>09_03.12.2024_Anregung_Ruecknahme_Beschwerde_DE_GH.pdf</t>
+          <t>10_12.12.2024_Hinweis_Beschwerde_und_eV_nur_schriftlich_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -901,36 +905,36 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>03.12.2024</t>
+          <t>12.12.2024</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Súd navrhuje späťvzatie sťažnosti (rozhodnutie z 21.11 doručené 26.11; sťažnosť z 25.11)</t>
+          <t>Súdny list: Beschwerde 07.12 a návrh na eV 11.12 prišli e-mailom, prípustné len písomne</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>→ klon P06</t>
+          <t>Súdny list (nie Petrov návrh na eV) → klon P10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Antrag_auf_Erlass_einer_einstweiligen_Verfugung_ORIGINAL_DE_GH.pdf</t>
+          <t>reklamacia_QES_zo_sudu_LA_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>10_12.12.2024_Hinweis_Beschwerde_und_eV_nur_schriftlich_DE_GH.pdf</t>
+          <t>11_17.12.2024_Hinweis_Form_par130a_Post_oder_QES_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -940,36 +944,36 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>12.12.2024</t>
+          <t>17.12.2024</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Súdny list: Beschwerde 07.12 a návrh na eV 11.12 prišli e-mailom, prípustné len písomne</t>
+          <t>Poučenie o forme § 130a: poštou s vlastnoručným podpisom ALEBO elektronicky s QES</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Súdny list (nie Petrov návrh na eV)</t>
+          <t>→ klon P11 (JADRO argumentu)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>reklamacia_QES_zo_sudu_LA_DE_GH.pdf</t>
+          <t>sud_LA_upozornenie_dokumenty_nepredstavuju_pravne_ucinne_navrhy_DE_original.pdf</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr"/>
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>11_17.12.2024_Hinweis_Form_par130a_Post_oder_QES_DE_GH.pdf</t>
+          <t>12_23.12.2024_Hinweis_Email_keine_formwirksamen_Antraege_nur_Post_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -979,36 +983,36 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>17.12.2024</t>
+          <t>23.12.2024</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Poučenie o forme § 130a: poštou s vlastnoručným podpisom ALEBO elektronicky s QES</t>
+          <t>E-maily nie sú formálne platné návrhy; kým nepodá poštou, e-maily sa už nebudú spracúvať</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>→ klon P03 (JADRO argumentu)</t>
+          <t>→ klon P12 (JADRO argumentu – odvolanie návodu)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>sud_LA_upozornenie_dokumenty_nepredstavuju_pravne_ucinne_navrhy_DE_original.pdf</t>
+          <t>sud_LA_zmena_spisovej_znacky_DE_GH.pdf</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>12_23.12.2024_Hinweis_Email_keine_formwirksamen_Antraege_nur_Post_DE_GH.pdf</t>
+          <t>13_07.01.2025_Aenderung_Aktenzeichen_91_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1018,36 +1022,36 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>23.12.2024</t>
+          <t>07.01.2025</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>E-maily nie sú formálne platné návrhy; kým nepodá poštou, e-maily sa už nebudú spracúvať</t>
+          <t>Zmena spisovej značky 23 O 2699/24 → 91 O 2699/24 (senát 526 → 416)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>→ klon P04 (JADRO argumentu – odvolanie návodu)</t>
+          <t>→ klon P13</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>sud_LA_zmena_spisovej_znacky_DE_GH.pdf</t>
+          <t>2025_01_22_LG_Landshut_potvrdenie_prijatia_emailu_20_01_2025_DE_original.pdf</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
       <c r="D14" s="3" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>13_07.01.2025_Aenderung_Aktenzeichen_91_O_2699_24_DE_GH.pdf</t>
+          <t>14_22.01.2025_Empfangsbestaetigung_Email_20_01_2025_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1057,58 +1061,19 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>07.01.2025</t>
+          <t>22.01.2025</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Zmena spisovej značky 23 O 2699/24 → 91 O 2699/24 (senát 526 → 416)</t>
+          <t>Potvrdenie prijatia e-mailu z 20.01.2025 (na sudcovský príkaz)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>→ klon P05</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>2025_01_22_LG_Landshut_potvrdenie_prijatia_emailu_20_01_2025_DE_original.pdf</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>14_22.01.2025_Empfangsbestaetigung_Email_20_01_2025_DE_GH.pdf</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>prijaté</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>22.01.2025</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Potvrdenie prijatia e-mailu z 20.01.2025 (na sudcovský príkaz)</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>→ klon P08; sken</t>
+          <t>→ klon P14; sken</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register prijate: precislovanie na suvisly rad 01-13 / P01-P13
</commit_message>
<xml_diff>
--- a/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
+++ b/sud-landshut-telekom/prijate/FIA_LG_Landshut_dokumenty_zoznam_prijate_GH.xlsx
@@ -763,7 +763,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -774,7 +774,7 @@
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>07_21.11.2024_Beschluss_PKH_beglaubigte_Abschrift_DE_GH.pdf</t>
+          <t>06_21.11.2024_Beschluss_PKH_beglaubigte_Abschrift_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -796,13 +796,13 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>→ klon P07; beglaubigte Abschrift (9 str.); originál Beschlussu 21.11 (06 zmazaný ako duplikát)</t>
+          <t>→ klon P06; beglaubigte Abschrift (9 str.); originál Beschlussu 21.11 (duplicitný „PKH abgelehnt" zmazaný)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>08_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
+          <t>07_27.11.2024_Kostennachricht_LJK_Bamberg_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -839,13 +839,13 @@
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>→ klon P08</t>
+          <t>→ klon P07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>09_03.12.2024_Anregung_Ruecknahme_Beschwerde_DE_GH.pdf</t>
+          <t>08_03.12.2024_Anregung_Ruecknahme_Beschwerde_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -878,13 +878,13 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>→ klon P09</t>
+          <t>→ klon P08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -895,7 +895,7 @@
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>10_12.12.2024_Hinweis_Beschwerde_und_eV_nur_schriftlich_DE_GH.pdf</t>
+          <t>09_12.12.2024_Hinweis_Beschwerde_und_eV_nur_schriftlich_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -917,13 +917,13 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Súdny list (nie Petrov návrh na eV) → klon P10</t>
+          <t>Súdny list (nie Petrov návrh na eV) → klon P09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -934,7 +934,7 @@
       <c r="D11" s="3" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>11_17.12.2024_Hinweis_Form_par130a_Post_oder_QES_DE_GH.pdf</t>
+          <t>10_17.12.2024_Hinweis_Form_par130a_Post_oder_QES_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -956,13 +956,13 @@
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>→ klon P11 (JADRO argumentu)</t>
+          <t>→ klon P10 (JADRO argumentu)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>12_23.12.2024_Hinweis_Email_keine_formwirksamen_Antraege_nur_Post_DE_GH.pdf</t>
+          <t>11_23.12.2024_Hinweis_Email_keine_formwirksamen_Antraege_nur_Post_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -995,13 +995,13 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>→ klon P12 (JADRO argumentu – odvolanie návodu)</t>
+          <t>→ klon P11 (JADRO argumentu – odvolanie návodu)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -1012,7 +1012,7 @@
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>13_07.01.2025_Aenderung_Aktenzeichen_91_O_2699_24_DE_GH.pdf</t>
+          <t>12_07.01.2025_Aenderung_Aktenzeichen_91_O_2699_24_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1034,13 +1034,13 @@
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>→ klon P13</t>
+          <t>→ klon P12</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1051,7 +1051,7 @@
       <c r="D14" s="3" t="inlineStr"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>14_22.01.2025_Empfangsbestaetigung_Email_20_01_2025_DE_GH.pdf</t>
+          <t>13_22.01.2025_Empfangsbestaetigung_Email_20_01_2025_DE_GH.pdf</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>→ klon P14; sken</t>
+          <t>→ klon P13; sken</t>
         </is>
       </c>
     </row>

</xml_diff>